<commit_message>
some more small tweaks
</commit_message>
<xml_diff>
--- a/details.xlsx
+++ b/details.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D666"/>
+  <dimension ref="A1:D755"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15068,6 +15068,1964 @@
         </is>
       </c>
     </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>65bd23ffa37c63bf8e185d1f</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>ShailabhRai</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>6388423228</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>https://d2bps9p1kiy4ka.cloudfront.net/5b09189f7285894d9130ccd0/621bfbec-aaa7-4e27-86e2-69c972ba1f14.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>641b0970c03bab034a895742</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>Mansi</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>7722884887</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>68123a0ed87791b53fe5e9b8</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>AbhishekKumar Roy</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>8409802174</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>62b035fb88440f00112f10c9</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>Saket Gupta</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>9519624242</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/ead93114-f600-480f-b394-f6ddba2dc81d.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>65f51777e8a07b574231624f</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>YuvrajBiru Singh</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>9227044118</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/729bcf01-8554-45f2-83ec-42eab0fac0d8.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>65941d8a5d5f62001870fdbb</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>Arpit Kumari</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>7061947946</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>https://d2bps9p1kiy4ka.cloudfront.net/5b09189f7285894d9130ccd0/7f57f875-5079-467b-8c7b-5a18589fc81c.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>67af562753a89f24529501dd</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>MuskanYadav</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>9608113147</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/16e387c1-89f1-4288-bd13-92a2a8dcfc8e.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>64ecf316270e74001858f7a8</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>PankajKumar</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>6206241709</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>6624d4c73ff1025bda82205a</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>VaibhavKhanderao</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>9011353494</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/e7c1e042-4cc3-4fcd-8b9c-d029ffb3275b.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>642bc5e7941d7b0018424441</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>Anjali</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>9155140066</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/9e7bdef5-f819-4ecf-8ec2-29493a057a44.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>69d753a71c7cbedc261e625d</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>Monika</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>7505633685</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/cfc3b52c-c05f-43ca-b85f-1bb29fa69cf6.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>650c52b04dd01c0018e387c9</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>YuktaSingh</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>8690840373</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>6a2ebc52bdf1d1e39cf87f53</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>NaziyaMulani</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>9665470130</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>62de77c28e48c1001848b61b</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>NaqueeReza</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>9510310785</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>https://d2bps9p1kiy4ka.cloudfront.net/5b09189f7285894d9130ccd0/4584bdbc-e32b-4bc7-8976-87d5df2ada3d.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>625be80584e9b6001173af6e</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>SachinKumar</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>7857933078</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/07359433-7962-4494-b7e3-d9677aa1227d.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>67f3bd1f62d1f60d454bbd16</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>SirMai Mai</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>7814030458</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/4d06a7ef-a7d1-4d08-b3c6-88ccd7e03f67.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>66d478702fd0c57d687171a0</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>PrashantSurya</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>9411742415</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>https://d2bps9p1kiy4ka.cloudfront.net/5b09189f7285894d9130ccd0/6595d91c-4fcf-4de1-acc4-8ceb3b5123b0.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>68dddf1505911a7d59cb14f2</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>SuryakantaSena</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>9124917192</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>6783bbbcb704ef4591159228</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>Zara</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>9336974073</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>6410ac78a20b8b001811ed39</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>Mishna</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>9508766612</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>6583273cf00b4b0018385552</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>KeshavKumar</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>7633966105</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/440bf2d8-9484-4932-9c12-eaf52ffd8e23.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>6303270d8a9e720018676893</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>XY</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>6005440768</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>69cd489cb7bb9d3b7e664f53</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>SimranRana</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>9528687391</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/8ce79d50-ecad-4138-b958-584aac4f50ff.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>65786e200b4d1f8b77cde699</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>SonalTomar</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>7879243623</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>https://d2bps9p1kiy4ka.cloudfront.net/5b09189f7285894d9130ccd0/8472137c-c044-49bf-a9fe-ff7beb3f3ff7.jfif</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>6738d2a3f581e947bf530698</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>DimpalSaraswat</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>9269985428</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>650733d7d912790018c6520c</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>Pranjal Rana</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>9244116516</t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/d6bfee33-a5c2-4cd5-b8dc-dd2e695f4e4b.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>67b821a4a365b1f3f334d39a</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>DeepDas</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>9957438211</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/30855a28-02e5-417c-b0d1-94224f51d28e.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>69cf38dcb7bb9d3b7e46e038</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>Rohit</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>8946926015</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/ad43cf9a-bc06-4c4f-97f7-54ac22a5543d.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>68014f7d34195dbe9cb68f3b</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>PriyanshuSingh</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>8797743837</t>
+        </is>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>64bca8d47d1f710018304ab6</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>Arjun</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>9418555302</t>
+        </is>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>663ccd1f62e0674fb798957f</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>Himanshiundefined</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>7503973563</t>
+        </is>
+      </c>
+      <c r="D697" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/e9bdac99-2268-49a3-acd3-860888367ae6.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>65ce1addb1b9d474d1bd3aae</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>PrateekCharan</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>7726872467</t>
+        </is>
+      </c>
+      <c r="D698" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/21539c9d-7ade-450f-afc0-f0b27cdfba3c.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>682afff103d3752aa3d5e8a8</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>AnushkaSwaraj</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>9795225825</t>
+        </is>
+      </c>
+      <c r="D699" t="inlineStr">
+        <is>
+          <t>https://d2bps9p1kiy4ka.cloudfront.net/5b09189f7285894d9130ccd0/1d137d13-da57-44a9-ad73-41f265a35de1.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>661fec742b5d15d4f0204e18</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>ShreyasiPal</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>9699570642</t>
+        </is>
+      </c>
+      <c r="D700" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>646aba9a2fc3810018c31a83</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>AiimsLovers</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>9006136478</t>
+        </is>
+      </c>
+      <c r="D701" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/7c6a2d8b-f4ac-4d7a-a28c-39622ee204ab.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>69db693c1c7cbedc26734c94</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>Jyoti</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>7235976494</t>
+        </is>
+      </c>
+      <c r="D702" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>641982c6f5df610018ee53de</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>Nishant</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>8955839231</t>
+        </is>
+      </c>
+      <c r="D703" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/4d1a3b50-27fc-4a3e-8166-77acdfd2e97c.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>689008338a2f4fa0c4c9ea6b</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>SushilKumar</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>7056860296</t>
+        </is>
+      </c>
+      <c r="D704" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/9e711a73-c9dc-4f23-a2e3-42d4bd859b48.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>66094d70ea39d2090aef5610</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>ArfajuddinAhammed</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>8972832055</t>
+        </is>
+      </c>
+      <c r="D705" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/ae187cb9-5926-45c4-aae4-d5490a18f1b1.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>6579489cd06c5500186309f0</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>RoshniSharma</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>8535032905</t>
+        </is>
+      </c>
+      <c r="D706" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>6437b7d477aac10018d199b9</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>DivyanshuRaj</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>9931479425</t>
+        </is>
+      </c>
+      <c r="D707" t="inlineStr">
+        <is>
+          <t>https://d2bps9p1kiy4ka.cloudfront.net/5b09189f7285894d9130ccd0/c7506bbc-21bd-4998-96a4-29b5bda4f67a.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>687991bbdbcbb76319bd70dd</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>Manasundefined</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>9509898592</t>
+        </is>
+      </c>
+      <c r="D708" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>66e1b5d9649668be9cc0e83f</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>ArsalaZulfiqar</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>7351397910</t>
+        </is>
+      </c>
+      <c r="D709" t="inlineStr">
+        <is>
+          <t>https://d2bps9p1kiy4ka.cloudfront.net/5b09189f7285894d9130ccd0/41e28be6-6760-4bdd-b0d3-b1425aeb96ab.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>6694d0dd5f25c67e2af6869c</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>Aditya</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>7014143889</t>
+        </is>
+      </c>
+      <c r="D710" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/a55a3002-fc8b-437a-8ca9-299966a8ecfd.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>6262ec7a46f38a00110bb21a</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>Vagisha</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>7458935936</t>
+        </is>
+      </c>
+      <c r="D711" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/ed5835a4-3f02-46e8-b4c6-8b60834845d9.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>66533e5adaa65a0019727bce</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>Tanisha Verma</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>9466891160</t>
+        </is>
+      </c>
+      <c r="D712" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/45071e8a-e77b-4b54-926d-727c6d4737e2.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>61d47e790f296d0011359a6d</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>AomJEE</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>9955604273</t>
+        </is>
+      </c>
+      <c r="D713" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>69facbb8a214ccc08a98da45</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>JapnoorSharma</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>9816478940</t>
+        </is>
+      </c>
+      <c r="D714" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/5bc03959-fcb6-4158-bc84-6cce33199aa6.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>65d0341b079e28936b76501d</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>VidzzzzzRaj</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>7209564571</t>
+        </is>
+      </c>
+      <c r="D715" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/b578ab81-8ca6-43f1-accd-34e6eb0d11ff.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>6531610b9dd3af001810e592</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>ShraddhaMishra</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>6393680499</t>
+        </is>
+      </c>
+      <c r="D716" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/2462fa9d-a843-4482-a86d-844cd3accdc3.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>667a7e358d05f008061abdf7</t>
+        </is>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>undefined</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>8918862979</t>
+        </is>
+      </c>
+      <c r="D717" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>685125c000168de99d02ff9c</t>
+        </is>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>AdarshTiwari</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>9555728284</t>
+        </is>
+      </c>
+      <c r="D718" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>667ff7637492c8528bda1672</t>
+        </is>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>DrVaishali</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>8350955884</t>
+        </is>
+      </c>
+      <c r="D719" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/e44a833e-c37a-4b50-938d-4659c278d9ad.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>641bec00b4c64c00181095f8</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>ArnabGhosh</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>8617525348</t>
+        </is>
+      </c>
+      <c r="D720" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/07d7c886-8576-4508-9548-366ced0340b3.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>640978dadd5a3b0019c1322b</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>Akash</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>9733618516</t>
+        </is>
+      </c>
+      <c r="D721" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>6605f781e685270018b1b68e</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>Nyasa Gangwarundefined</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>8318729612</t>
+        </is>
+      </c>
+      <c r="D722" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/6d8ae63a-3698-4b8d-a97b-9773e7ea671c.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>63e7b703ad096e02c9fae217</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>Sonu</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>7838663835</t>
+        </is>
+      </c>
+      <c r="D723" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>663b10cc67a0d86bd6f6f47c</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>PrachiSingh</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>6386079894</t>
+        </is>
+      </c>
+      <c r="D724" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>65bb667dd06ce78304966fb1</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>SunilKr Singh</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>6388708970</t>
+        </is>
+      </c>
+      <c r="D725" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/49345cf5-aca3-4f82-9819-53df006e4e3a.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>625ac85e0febd70015b937c0</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>SrishtiVerma Kala Upadhyay</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>9161858431</t>
+        </is>
+      </c>
+      <c r="D726" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>6876cfdb66f14e5c5ea48fb7</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>Khushiundefined</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>9389747438</t>
+        </is>
+      </c>
+      <c r="D727" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>65785f3fa957170019e08f25</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>ShreyaPatel</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>7307889334</t>
+        </is>
+      </c>
+      <c r="D728" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/256acc3b-873a-4d5e-986e-52fca018eb2c.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>64faf9a9f0fa33001829dcf7</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>MahimaKumari</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>9119753035</t>
+        </is>
+      </c>
+      <c r="D729" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>660bab1deb6c7500180478d3</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>KamranKhan</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>8115201646</t>
+        </is>
+      </c>
+      <c r="D730" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/3423579e-7857-481f-9b79-9c101ce0eb46.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>63ae9020b43ec00012693186</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>UtsavKaghariya</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>9340276823</t>
+        </is>
+      </c>
+      <c r="D731" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/8e58efc8-aba5-45b4-be04-7a7024b2d77b.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>635aa4432c726f001102ee11</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>Anmolnayak</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>7752937913</t>
+        </is>
+      </c>
+      <c r="D732" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>6a036be12db7465a85ad4557</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>Muskan</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>8169669576</t>
+        </is>
+      </c>
+      <c r="D733" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>68289be403d3752aa3db009b</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>Sneha</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>8459775166</t>
+        </is>
+      </c>
+      <c r="D734" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/893286a5-7a05-4384-920a-03c2319226b5.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>641bbbc2a40b5700189e499d</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>NeverGive Up</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>6394360477</t>
+        </is>
+      </c>
+      <c r="D735" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/b7ce2bf6-8d2c-44c6-9086-6186ca97ef66.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>682d4f9103d3752aa3302143</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>TabishJafri</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>9263600454</t>
+        </is>
+      </c>
+      <c r="D736" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/fab36082-9d72-4f8f-9d88-816f94a0bcc9.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>62a4ba938260e10018d95812</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>Punyasharma</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>8900092179</t>
+        </is>
+      </c>
+      <c r="D737" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>65091f29df04420018fe8c84</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>Mohit</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>9797494085</t>
+        </is>
+      </c>
+      <c r="D738" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/8a214f04-d86a-4db5-9c60-c8aa5376a898.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>69a9a5f20d2994f1713cbce3</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>ArpanYadav</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>8676044926</t>
+        </is>
+      </c>
+      <c r="D739" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/136e4420-affa-46b5-8428-128a0b039400.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>675927834f3b1179b4995f83</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>AshnaNag</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>9122572912</t>
+        </is>
+      </c>
+      <c r="D740" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/0910bdcf-cf22-4f74-abad-345298b35c7a.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>6a01c107a214ccc08a2bba88</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>Ayushi</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>7889661550</t>
+        </is>
+      </c>
+      <c r="D741" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>64c491b9e325a3001811c122</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>SagarRajput</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>9098060843</t>
+        </is>
+      </c>
+      <c r="D742" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>6a4921ab446b978db06a6b54</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>AryanSharma</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>9306314889</t>
+        </is>
+      </c>
+      <c r="D743" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>678a459c77a19983dca93aa5</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>DibyajyotiMallick</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>9733427947</t>
+        </is>
+      </c>
+      <c r="D744" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>649c52af3a0b150018f0eb83</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>JyotirmayaTandi</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>7751969512</t>
+        </is>
+      </c>
+      <c r="D745" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/75e1b934-92d6-44b1-aa7e-f6dd1679e026.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>62931597e96184001830488d</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>AnjaliDahariya</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>7879590693</t>
+        </is>
+      </c>
+      <c r="D746" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/ff862245-8f95-48fa-8cae-b2d7e923a89c.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>67b0c02253a89f24521af9df</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>TanuSingh</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>6397164273</t>
+        </is>
+      </c>
+      <c r="D747" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/392b2cac-9439-4188-8559-5704163f53de.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>6a42217b446b978db04b91ed</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>SanjayGurjar</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>8690014650</t>
+        </is>
+      </c>
+      <c r="D748" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>65e86a42cea7400018f4a855</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>MdDanish</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>9817228037</t>
+        </is>
+      </c>
+      <c r="D749" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/bc437f77-1b3a-46ae-9edf-bf9a2919472e.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>665601165104a911f3b69623</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>SuluuuuuuuuuuHuluuuuuuuuuuuuuuuuuuuu</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>7261887573</t>
+        </is>
+      </c>
+      <c r="D750" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/804851fc-70ce-411a-88bb-e78ad6871441.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>65cb0f0871cc9100184a8412</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>ShreyaAiims</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>6294984391</t>
+        </is>
+      </c>
+      <c r="D751" t="inlineStr">
+        <is>
+          <t>https://d2bps9p1kiy4ka.cloudfront.net/5b09189f7285894d9130ccd0/be740135-c54c-4c3c-90e2-e88c7520d49e.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>67489443514982cb6bee9736</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>PritamKumar</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>7061050923</t>
+        </is>
+      </c>
+      <c r="D752" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>647df27acffdde00185ee3fd</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>MemeBoy</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>7905421200</t>
+        </is>
+      </c>
+      <c r="D753" t="inlineStr">
+        <is>
+          <t>https://d2bps9p1kiy4ka.cloudfront.net/5b09189f7285894d9130ccd0/2d6117b4-768e-4487-9d97-ad7283c6dec0.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>64d0d9e58d96a700181a1162</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>ShauryaSingh</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>9473056092</t>
+        </is>
+      </c>
+      <c r="D754" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5b09189f7285894d9130ccd0/a96eb535-d433-4398-aabe-c5413a48ead1.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>6937c9db419480a39e24a4db</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>SurajSawant</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>8261879011</t>
+        </is>
+      </c>
+      <c r="D755" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>